<commit_message>
refactor: update task configuration, remove legacy CBAC referral forms, and add new high-risk and PHQ2 referral forms.
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/phq9.xlsx
+++ b/config/demo/forms/app/phq9.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I118"/>
+  <dimension ref="I1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="8" min="1" max="1"/>
@@ -667,24 +667,24 @@
     <row r="14" ht="15" customHeight="1" s="9">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>cbac_source_id</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="9">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>user</t>
         </is>
       </c>
     </row>
@@ -696,83 +696,63 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>name</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="9">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>phone</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="9">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>reporter_name_note</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Filled by: ${reporter_name}</t>
+          <t>user</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="9">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>contact</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n"/>
+          <t>reporter_name_note</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Filled by: ${reporter_name}</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="9">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>_id</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Patient's Name</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Select the patient from your area</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>select-contact type-patient</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="9">
       <c r="A21" s="8" t="inlineStr">
@@ -782,17 +762,27 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>_id</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Medic ID</t>
+          <t>Patient's Name</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Select the patient from your area</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>select-contact type-patient</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -804,12 +794,12 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Patient Name</t>
+          <t>Medic ID</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -821,56 +811,51 @@
     <row r="23" ht="15" customHeight="1" s="9">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>string</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>hidden</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="9">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>select_one states</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>contact</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="9">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>select_one districts</t>
+          <t>select_one states</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>District</t>
+          <t>State</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -881,57 +866,67 @@
       <c r="G25" s="8" t="inlineStr">
         <is>
           <t>yes</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>filter = ${state}</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="9">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one districts</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>inputs</t>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>filter = ${state}</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="9">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>instructions</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>inputs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="9">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>instructions_1</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PHQ-9: Patient Health Questionnaire  </t>
+          <t>instructions</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -943,12 +938,12 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Instructions_2</t>
+          <t>instructions_1</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Over the last 2 weeks, how often have you been bothered by any of the following problems? Answer all 9 questions. Each question is scored: </t>
+          <t xml:space="preserve">PHQ-9: Patient Health Questionnaire  </t>
         </is>
       </c>
     </row>
@@ -960,12 +955,12 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Instructions_3</t>
+          <t>Instructions_2</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Not at all=0,</t>
+          <t xml:space="preserve">Over the last 2 weeks, how often have you been bothered by any of the following problems? Answer all 9 questions. Each question is scored: </t>
         </is>
       </c>
     </row>
@@ -977,12 +972,12 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Instructions_4</t>
+          <t>Instructions_3</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Several days=1, </t>
+          <t>Not at all=0,</t>
         </is>
       </c>
     </row>
@@ -994,12 +989,12 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Instructions_5</t>
+          <t>Instructions_4</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">More than half the days=2, </t>
+          <t xml:space="preserve">Several days=1, </t>
         </is>
       </c>
     </row>
@@ -1011,74 +1006,64 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Instructions_6</t>
+          <t>Instructions_5</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Nearly every day=3</t>
+          <t xml:space="preserve">More than half the days=2, </t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="9">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>instructions</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n"/>
+          <t>Instructions_6</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Nearly every day=3</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="9">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>page_1</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Questions 1 &amp; 2 of 9</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+          <t>instructions</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="9">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>little_interest_or_pleasure</t>
+          <t>page_1</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>1. Little interest or pleasure in doing things</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Use ✓ to indicate your answer</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Questions 1 &amp; 2 of 9</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1075,12 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>feeling_depressed_or_hopeless</t>
+          <t>little_interest_or_pleasure</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>2. Feeling down, depressed, or hopeless</t>
+          <t>1. Little interest or pleasure in doing things</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -1112,61 +1097,61 @@
     <row r="38" ht="15" customHeight="1" s="9">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>page_1</t>
+          <t>feeling_depressed_or_hopeless</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>2. Feeling down, depressed, or hopeless</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Use ✓ to indicate your answer</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="9">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>page_2</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Questions 3 &amp; 4 of 9</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>page_1</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="9">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>trouble_sleeping</t>
+          <t>page_2</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>3. Trouble falling or staying asleep, or sleeping too much</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Use ✓ to indicate your answer</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Questions 3 &amp; 4 of 9</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1163,12 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>feeling_tired</t>
+          <t>trouble_sleeping</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>4. Feeling tired or having little energy</t>
+          <t>3. Trouble falling or staying asleep, or sleeping too much</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -1200,61 +1185,61 @@
     <row r="42" ht="15" customHeight="1" s="9">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>page_2</t>
+          <t>feeling_tired</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>4. Feeling tired or having little energy</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Use ✓ to indicate your answer</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="9">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>page_3</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Questions 5 &amp; 6 of 9</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>page_2</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="9">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>poor_appetite_or_overeating</t>
+          <t>page_3</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>5. Poor appetite or overeating</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Use ✓ to indicate your answer</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Questions 5 &amp; 6 of 9</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1251,12 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>feeling_bad_about_yourself</t>
+          <t>poor_appetite_or_overeating</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>6. Feeling bad about yourself — or that you are a failure or have let yourself or your family down</t>
+          <t>5. Poor appetite or overeating</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -1288,61 +1273,61 @@
     <row r="46" ht="15" customHeight="1" s="9">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>page_3</t>
+          <t>feeling_bad_about_yourself</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>6. Feeling bad about yourself — or that you are a failure or have let yourself or your family down</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Use ✓ to indicate your answer</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="9">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>page_4</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Questions 7 &amp; 8 of 9</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>page_3</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>trouble_concentrating</t>
+          <t>page_4</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>7. Trouble concentrating on things, such as reading the newspaper or watching television</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Use ✓ to indicate your answer</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Questions 7 &amp; 8 of 9</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
@@ -1354,12 +1339,12 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>moving_or_speaking_slowly</t>
+          <t>trouble_concentrating</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>8. Moving or speaking so slowly that other people could have noticed? Or the opposite — being so fidgety or restless that you have been moving around a lot more than usual</t>
+          <t>7. Trouble concentrating on things, such as reading the newspaper or watching television</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -1376,90 +1361,100 @@
     <row r="50" ht="15" customHeight="1" s="9">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>page_4</t>
+          <t>moving_or_speaking_slowly</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>8. Moving or speaking so slowly that other people could have noticed? Or the opposite — being so fidgety or restless that you have been moving around a lot more than usual</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Use ✓ to indicate your answer</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="9">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>page_5</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Question 9 of 9</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>page_4</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="9">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>select_one frequency</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>thoughts_of_self_harm</t>
+          <t>page_5</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>9. Thoughts that you would be better off dead or of hurting yourself in some way</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Use ✓ to indicate your answer</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Question 9 of 9</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="9">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>select_one frequency</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>page_5</t>
+          <t>thoughts_of_self_harm</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>9. Thoughts that you would be better off dead or of hurting yourself in some way</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Use ✓ to indicate your answer</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="9">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>total_score</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>${little_interest_or_pleasure} + ${feeling_depressed_or_hopeless} + ${trouble_sleeping} + ${feeling_tired} + ${poor_appetite_or_overeating} + ${feeling_bad_about_yourself} + ${trouble_concentrating} + ${moving_or_speaking_slowly} + ${thoughts_of_self_harm}</t>
+          <t>page_5</t>
         </is>
       </c>
     </row>
@@ -1471,34 +1466,29 @@
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>severity_category</t>
+          <t>total_score</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>if(${total_score} &lt;= 4, 'minimal', if(${total_score} &lt;= 9, 'mild', if(${total_score} &lt;= 14, 'moderate', if(${total_score} &lt;= 19, 'moderately_severe', 'severe'))))</t>
+          <t>${little_interest_or_pleasure} + ${feeling_depressed_or_hopeless} + ${trouble_sleeping} + ${feeling_tired} + ${poor_appetite_or_overeating} + ${feeling_bad_about_yourself} + ${trouble_concentrating} + ${moving_or_speaking_slowly} + ${thoughts_of_self_harm}</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="9">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>group_summary</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>Assessment Summary for Mental Health Form</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>severity_category</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>if(${total_score} &lt;= 4, 'minimal', if(${total_score} &lt;= 9, 'mild', if(${total_score} &lt;= 14, 'moderate', if(${total_score} &lt;= 19, 'moderately_severe', 'severe'))))</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1500,12 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_filled_by</t>
+          <t>group_summary</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Assessment Summary for Mental Health Form</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -1522,967 +1517,984 @@
     <row r="58" ht="15" customHeight="1" s="9">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>lbl_filled_by_lbl</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>**Filled by:**  ${reporter_name}</t>
+          <t>grp_lbl_filled_by</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="9">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>calc_reporter_name</t>
-        </is>
-      </c>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>${reporter_name}</t>
+          <t>lbl_filled_by_lbl</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>**Filled by:**  ${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="9">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_filled_by</t>
+          <t>calc_reporter_name</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>${reporter_name}</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="9">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_patient</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_filled_by</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="9">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>lbl_patient_lbl</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>**Patient:**  ${patient_name}</t>
+          <t>grp_lbl_patient</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="9">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>calc_patient_name</t>
-        </is>
-      </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>${patient_name}</t>
+          <t>lbl_patient_lbl</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>**Patient:**  ${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="9">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_patient</t>
+          <t>calc_patient_name</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>${patient_name}</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="9">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_state</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_patient</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="9">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>lbl_state_lbl</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>**State:**  ${calc_state}</t>
+          <t>grp_lbl_state</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="9">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>calc_state</t>
-        </is>
-      </c>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${state}, '${state}')</t>
+          <t>lbl_state_lbl</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>**State:**  ${calc_state}</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="9">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_state</t>
+          <t>calc_state</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${state}, '${state}')</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="9">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_district</t>
-        </is>
-      </c>
-      <c r="E69" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_state</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="9">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>lbl_district_lbl</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>**District:**  ${calc_district}</t>
+          <t>grp_lbl_district</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="9">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>calc_district</t>
-        </is>
-      </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${district}, '${district}')</t>
+          <t>lbl_district_lbl</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>**District:**  ${calc_district}</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="9">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_district</t>
+          <t>calc_district</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${district}, '${district}')</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="9">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q1</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_district</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="9">
       <c r="A74" s="8" t="inlineStr">
         <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>grp_lbl_q1</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15" customHeight="1" s="9">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>lbl_q1_lbl</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>**1. Little interest or pleasure in doing things:** ${calc_q1}</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="15.75" customHeight="1" s="9">
-      <c r="A75" s="8" t="inlineStr">
+    <row r="76" ht="15.75" customHeight="1" s="9">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>calculate</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>calc_q1</t>
         </is>
       </c>
-      <c r="F75" s="8" t="inlineStr">
+      <c r="F76" s="8" t="inlineStr">
         <is>
           <t>jr:choice-name(${little_interest_or_pleasure}, '${little_interest_or_pleasure}')</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="15" customHeight="1" s="9">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>grp_lbl_q1</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="9">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q2</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q1</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="9">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>lbl_q2_lbl</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>**2. Feeling down, depressed, or hopeless:** ${calc_q2}</t>
+          <t>grp_lbl_q2</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="9">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>calc_q2</t>
-        </is>
-      </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${feeling_depressed_or_hopeless}, '${feeling_depressed_or_hopeless}')</t>
+          <t>lbl_q2_lbl</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>**2. Feeling down, depressed, or hopeless:** ${calc_q2}</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="9">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q2</t>
+          <t>calc_q2</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${feeling_depressed_or_hopeless}, '${feeling_depressed_or_hopeless}')</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="9">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q3</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q2</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="9">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>lbl_q3_lbl</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>**3. Trouble falling or staying asleep, or sleeping too much:** ${calc_q3}</t>
+          <t>grp_lbl_q3</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="9">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>calc_q3</t>
-        </is>
-      </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${trouble_sleeping}, '${trouble_sleeping}')</t>
+          <t>lbl_q3_lbl</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>**3. Trouble falling or staying asleep, or sleeping too much:** ${calc_q3}</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="9">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q3</t>
+          <t>calc_q3</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${trouble_sleeping}, '${trouble_sleeping}')</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="9">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q4</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q3</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="9">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>lbl_q4_lbl</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>**4. Feeling tired or having little energy:** ${calc_q4}</t>
+          <t>grp_lbl_q4</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="9">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>calc_q4</t>
-        </is>
-      </c>
-      <c r="F87" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${feeling_tired}, '${feeling_tired}')</t>
+          <t>lbl_q4_lbl</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>**4. Feeling tired or having little energy:** ${calc_q4}</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="9">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q4</t>
+          <t>calc_q4</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${feeling_tired}, '${feeling_tired}')</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="9">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q5</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q4</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="9">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>lbl_q5_lbl</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>**5. Poor appetite or overeating:** ${calc_q5}</t>
+          <t>grp_lbl_q5</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="9">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>calc_q5</t>
-        </is>
-      </c>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${poor_appetite_or_overeating}, '${poor_appetite_or_overeating}')</t>
+          <t>lbl_q5_lbl</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>**5. Poor appetite or overeating:** ${calc_q5}</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="9">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q5</t>
+          <t>calc_q5</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${poor_appetite_or_overeating}, '${poor_appetite_or_overeating}')</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="9">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q6</t>
-        </is>
-      </c>
-      <c r="E93" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q5</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="9">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>lbl_q6_lbl</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t>**6. Feeling bad about yourself — or that you are a failure or have let yourself or your family down:** ${calc_q6}</t>
+          <t>grp_lbl_q6</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="9">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>calc_q6</t>
-        </is>
-      </c>
-      <c r="F95" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${feeling_bad_about_yourself}, '${feeling_bad_about_yourself}')</t>
+          <t>lbl_q6_lbl</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>**6. Feeling bad about yourself — or that you are a failure or have let yourself or your family down:** ${calc_q6}</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="9">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q6</t>
+          <t>calc_q6</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${feeling_bad_about_yourself}, '${feeling_bad_about_yourself}')</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="9">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q7</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q6</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="9">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>lbl_q7_lbl</t>
-        </is>
-      </c>
-      <c r="C98" s="8" t="inlineStr">
-        <is>
-          <t>**7. Trouble concentrating on things, such as reading the newspaper or watching television:** ${calc_q7}</t>
+          <t>grp_lbl_q7</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="9">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>calc_q7</t>
-        </is>
-      </c>
-      <c r="F99" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${trouble_concentrating}, '${trouble_concentrating}')</t>
+          <t>lbl_q7_lbl</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>**7. Trouble concentrating on things, such as reading the newspaper or watching television:** ${calc_q7}</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="9">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q7</t>
+          <t>calc_q7</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${trouble_concentrating}, '${trouble_concentrating}')</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="9">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q8</t>
-        </is>
-      </c>
-      <c r="E101" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q7</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="9">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>lbl_q8_lbl</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>**8. Moving or speaking so slowly that other people could have noticed? Or the opposite — being so fidgety or restless that you have been moving around a lot more than usual:** ${calc_q8}</t>
+          <t>grp_lbl_q8</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="9">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>calc_q8</t>
-        </is>
-      </c>
-      <c r="F103" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${moving_or_speaking_slowly}, '${moving_or_speaking_slowly}')</t>
+          <t>lbl_q8_lbl</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>**8. Moving or speaking so slowly that other people could have noticed? Or the opposite — being so fidgety or restless that you have been moving around a lot more than usual:** ${calc_q8}</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="9">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q8</t>
+          <t>calc_q8</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${moving_or_speaking_slowly}, '${moving_or_speaking_slowly}')</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="9">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q9</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q8</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="9">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>lbl_q9_lbl</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="inlineStr">
-        <is>
-          <t>**9. Thoughts that you would be better off dead or of hurting yourself in some way:** ${calc_q9}</t>
+          <t>grp_lbl_q9</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="9">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>calc_q9</t>
-        </is>
-      </c>
-      <c r="F107" s="8" t="inlineStr">
-        <is>
-          <t>jr:choice-name(${thoughts_of_self_harm}, '${thoughts_of_self_harm}')</t>
+          <t>lbl_q9_lbl</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>**9. Thoughts that you would be better off dead or of hurting yourself in some way:** ${calc_q9}</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="9">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_q9</t>
+          <t>calc_q9</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>jr:choice-name(${thoughts_of_self_harm}, '${thoughts_of_self_harm}')</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="9">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_score</t>
-        </is>
-      </c>
-      <c r="E109" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_q9</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="9">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>lbl_score_lbl</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
-          <t>**PHQ-9 Total Score:**  ${total_score} / 27</t>
+          <t>grp_lbl_score</t>
+        </is>
+      </c>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="9">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>calc_total_score</t>
-        </is>
-      </c>
-      <c r="F111" s="8" t="inlineStr">
-        <is>
-          <t>${total_score}</t>
+          <t>lbl_score_lbl</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>**PHQ-9 Total Score:**  ${total_score} / 27</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="9">
       <c r="A112" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_score</t>
+          <t>calc_total_score</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>${total_score}</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="9">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t>begin group</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_severity</t>
-        </is>
-      </c>
-      <c r="E113" s="8" t="inlineStr">
-        <is>
-          <t>field-list</t>
+          <t>grp_lbl_score</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="9">
       <c r="A114" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>lbl_severity_lbl</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t>**Severity:**  ${calc_severity_category}</t>
+          <t>grp_lbl_severity</t>
+        </is>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>field-list</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="9">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>calc_severity_category</t>
-        </is>
-      </c>
-      <c r="F115" s="8" t="inlineStr">
-        <is>
-          <t>if(${severity_category} = 'minimal', 'Minimal (0–4)', if(${severity_category} = 'mild', 'Mild (5–9)', if(${severity_category} = 'moderate', 'Moderate (10–14)', if(${severity_category} = 'moderately_severe', 'Moderately Severe (15–19)', if(${severity_category} = 'severe', 'Severe (20–27)', ${severity_category})))))</t>
+          <t>lbl_severity_lbl</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>**Severity:**  ${calc_severity_category}</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="9">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>end group</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>grp_lbl_severity</t>
+          <t>calc_severity_category</t>
+        </is>
+      </c>
+      <c r="F116" s="8" t="inlineStr">
+        <is>
+          <t>if(${severity_category} = 'minimal', 'Minimal (0–4)', if(${severity_category} = 'mild', 'Mild (5–9)', if(${severity_category} = 'moderate', 'Moderate (10–14)', if(${severity_category} = 'moderately_severe', 'Moderately Severe (15–19)', if(${severity_category} = 'severe', 'Severe (20–27)', ${severity_category})))))</t>
         </is>
       </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="9">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>end group</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>severity_guide</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>0–4 Minimal  ·  5–9 Mild  ·  10–14 Moderate  ·  15–19 Mod. Severe  ·  20–27 Severe</t>
+          <t>grp_lbl_severity</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="9">
       <c r="A118" s="8" t="inlineStr">
         <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>severity_guide</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>0–4 Minimal  ·  5–9 Mild  ·  10–14 Moderate  ·  15–19 Mod. Severe  ·  20–27 Severe</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15" customHeight="1" s="9">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B118" s="8" t="inlineStr">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t>group_summary</t>
         </is>
       </c>
     </row>
-    <row r="1048570" ht="12.75" customHeight="1" s="9"/>
     <row r="1048571" ht="12.75" customHeight="1" s="9"/>
     <row r="1048572" ht="12.75" customHeight="1" s="9"/>
     <row r="1048573" ht="12.75" customHeight="1" s="9"/>
     <row r="1048574" ht="12.75" customHeight="1" s="9"/>
     <row r="1048575" ht="12.75" customHeight="1" s="9"/>
     <row r="1048576" ht="12.75" customHeight="1" s="9"/>
+    <row r="1048577" ht="12.75" customHeight="1" s="9"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>